<commit_message>
feat: complete PostgreSQL database redesign
- Redesign the persistence model into a 13-table PostgreSQL schema
- Add ERD v1.2, seed data, constraint tests, and migration documentation
- Migrate DAO persistence SQL from Oracle-specific syntax to PostgreSQL
- Normalize test scores into correct_count and total_count
- Preserve makeup scheduling through a nullable target_lesson_id foreign key
- Add message delivery and import audit history models
- Introduce SHA-256 file and row tracking without storing duplicate raw row payloads in audit tables
- Update sample data, configuration examples, automated tests, and project documentation
</commit_message>
<xml_diff>
--- a/data/sample_students.xlsx
+++ b/data/sample_students.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="R23d76924101c4726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="Rfbeea00e20e34a95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,10 +458,8 @@
           <x:t xml:space="preserve">B</x:t>
         </x:is>
       </x:c>
-      <x:c r="M2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">85점</x:t>
-        </x:is>
+      <x:c r="M2" t="str">
+        <x:v>13/39</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -568,10 +566,8 @@
           <x:t xml:space="preserve">A</x:t>
         </x:is>
       </x:c>
-      <x:c r="M4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">92점</x:t>
-        </x:is>
+      <x:c r="M4" t="str">
+        <x:v>39/50</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>